<commit_message>
Changed song names in excel
changed the names of folklore and evermore in excel to match the database
</commit_message>
<xml_diff>
--- a/excelToJS/taylor_all_album_songs.xlsx
+++ b/excelToJS/taylor_all_album_songs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stormwinnem/Desktop/Repositories/Swift-Sounds/excelToJS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98672B2B-BF17-B740-9AA6-C2ECEAF270AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{761BA1E9-4E62-824F-86B8-8564E25A13B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{0842053E-6FEE-2E43-A668-BC17E9E71A07}"/>
   </bookViews>
@@ -333,9 +333,6 @@
     <t>Daylight</t>
   </si>
   <si>
-    <t>folklore</t>
-  </si>
-  <si>
     <t>the 1</t>
   </si>
   <si>
@@ -381,9 +378,6 @@
     <t>hoax</t>
   </si>
   <si>
-    <t>evermore</t>
-  </si>
-  <si>
     <t>willow</t>
   </si>
   <si>
@@ -817,6 +811,12 @@
   </si>
   <si>
     <t>Midnights (The Til Dawn Edition)</t>
+  </si>
+  <si>
+    <t>evermore (deluxe version)</t>
+  </si>
+  <si>
+    <t>folklore (deluxe version)</t>
   </si>
 </sst>
 </file>
@@ -1246,7 +1246,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B3">
         <v>2</v>
@@ -1272,20 +1272,20 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B4">
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B5">
         <v>4</v>
@@ -1297,7 +1297,7 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B6">
         <v>5</v>
@@ -1309,7 +1309,7 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B7">
         <v>6</v>
@@ -1321,7 +1321,7 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B8">
         <v>7</v>
@@ -1333,7 +1333,7 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B9">
         <v>8</v>
@@ -1345,7 +1345,7 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B10">
         <v>9</v>
@@ -1358,7 +1358,7 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B11">
         <v>10</v>
@@ -1370,7 +1370,7 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B12">
         <v>11</v>
@@ -1383,7 +1383,7 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B13">
         <v>12</v>
@@ -1395,7 +1395,7 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B14">
         <v>13</v>
@@ -1407,7 +1407,7 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B15">
         <v>14</v>
@@ -1419,13 +1419,13 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B16">
         <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K16" s="1"/>
     </row>
@@ -1510,7 +1510,7 @@
         <v>7</v>
       </c>
       <c r="C23" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="K23" s="1"/>
     </row>
@@ -1618,7 +1618,7 @@
         <v>16</v>
       </c>
       <c r="C32" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="K32" s="1"/>
     </row>
@@ -1678,7 +1678,7 @@
         <v>21</v>
       </c>
       <c r="C37" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="I37" s="1"/>
       <c r="K37" s="1"/>
@@ -1691,7 +1691,7 @@
         <v>22</v>
       </c>
       <c r="C38" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I38" s="1"/>
       <c r="K38" s="1"/>
@@ -1704,7 +1704,7 @@
         <v>23</v>
       </c>
       <c r="C39" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="K39" s="1"/>
     </row>
@@ -1716,7 +1716,7 @@
         <v>24</v>
       </c>
       <c r="C40" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="K40" s="1"/>
     </row>
@@ -1728,7 +1728,7 @@
         <v>25</v>
       </c>
       <c r="C41" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="K41" s="1"/>
     </row>
@@ -1740,45 +1740,45 @@
         <v>26</v>
       </c>
       <c r="C42" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="K42" s="1"/>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B43">
         <v>1</v>
       </c>
       <c r="C43" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="J43" s="1"/>
       <c r="K43" s="1"/>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B44">
         <v>2</v>
       </c>
       <c r="C44" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="J44" s="1"/>
       <c r="K44" s="1"/>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B45">
         <v>3</v>
       </c>
       <c r="C45" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="I45" s="1"/>
       <c r="J45" s="1"/>
@@ -1786,38 +1786,38 @@
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B46">
         <v>4</v>
       </c>
       <c r="C46" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="I46" s="1"/>
       <c r="K46" s="1"/>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B47">
         <v>5</v>
       </c>
       <c r="C47" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="K47" s="1"/>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B48">
         <v>6</v>
       </c>
       <c r="C48" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="I48" s="1"/>
       <c r="J48" s="1"/>
@@ -1825,197 +1825,197 @@
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B49">
         <v>7</v>
       </c>
       <c r="C49" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="J49" s="1"/>
       <c r="K49" s="1"/>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B50">
         <v>8</v>
       </c>
       <c r="C50" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="K50" s="1"/>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B51">
         <v>9</v>
       </c>
       <c r="C51" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="K51" s="1"/>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B52">
         <v>10</v>
       </c>
       <c r="C52" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K52" s="1"/>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B53">
         <v>11</v>
       </c>
       <c r="C53" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="K53" s="1"/>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B54">
         <v>12</v>
       </c>
       <c r="C54" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="K54" s="1"/>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B55">
         <v>13</v>
       </c>
       <c r="C55" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="K55" s="1"/>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B56">
         <v>14</v>
       </c>
       <c r="C56" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="K56" s="1"/>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B57">
         <v>15</v>
       </c>
       <c r="C57" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="J57" s="1"/>
       <c r="K57" s="1"/>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B58">
         <v>16</v>
       </c>
       <c r="C58" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="I58" s="1"/>
       <c r="K58" s="1"/>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B59">
         <v>17</v>
       </c>
       <c r="C59" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="I59" s="1"/>
       <c r="K59" s="1"/>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B60">
         <v>18</v>
       </c>
       <c r="C60" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K60" s="1"/>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B61">
         <v>19</v>
       </c>
       <c r="C61" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="K61" s="1"/>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B62">
         <v>20</v>
       </c>
       <c r="C62" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="K62" s="1"/>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B63">
         <v>21</v>
       </c>
       <c r="C63" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="K63" s="1"/>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B64">
         <v>22</v>
       </c>
       <c r="C64" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="K64" s="1"/>
     </row>
@@ -2135,7 +2135,7 @@
         <v>10</v>
       </c>
       <c r="C74" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="K74" s="1"/>
     </row>
@@ -2183,7 +2183,7 @@
         <v>14</v>
       </c>
       <c r="C78" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="K78" s="1"/>
     </row>
@@ -2255,7 +2255,7 @@
         <v>20</v>
       </c>
       <c r="C84" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="K84" s="1"/>
     </row>
@@ -2279,7 +2279,7 @@
         <v>22</v>
       </c>
       <c r="C86" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="K86" s="1"/>
     </row>
@@ -2291,7 +2291,7 @@
         <v>23</v>
       </c>
       <c r="C87" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="K87" s="1"/>
     </row>
@@ -2303,7 +2303,7 @@
         <v>24</v>
       </c>
       <c r="C88" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="K88" s="1"/>
     </row>
@@ -2315,7 +2315,7 @@
         <v>25</v>
       </c>
       <c r="C89" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="I89" s="1"/>
       <c r="K89" s="1"/>
@@ -2328,7 +2328,7 @@
         <v>26</v>
       </c>
       <c r="C90" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="I90" s="1"/>
       <c r="K90" s="1"/>
@@ -2341,7 +2341,7 @@
         <v>27</v>
       </c>
       <c r="C91" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="J91" s="1"/>
       <c r="K91" s="1"/>
@@ -2354,7 +2354,7 @@
         <v>28</v>
       </c>
       <c r="C92" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="J92" s="1"/>
       <c r="K92" s="1"/>
@@ -2367,7 +2367,7 @@
         <v>29</v>
       </c>
       <c r="C93" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="I93" s="1"/>
       <c r="J93" s="1"/>
@@ -2381,142 +2381,142 @@
         <v>30</v>
       </c>
       <c r="C94" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="K94" s="1"/>
     </row>
     <row r="95" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B95">
         <v>1</v>
       </c>
       <c r="C95" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="J95" s="1"/>
       <c r="K95" s="1"/>
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B96">
         <v>2</v>
       </c>
       <c r="C96" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="K96" s="1"/>
     </row>
     <row r="97" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B97">
         <v>3</v>
       </c>
       <c r="C97" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="K97" s="1"/>
     </row>
     <row r="98" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B98">
         <v>4</v>
       </c>
       <c r="C98" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="J98" s="1"/>
       <c r="K98" s="1"/>
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B99">
         <v>5</v>
       </c>
       <c r="C99" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="K99" s="1"/>
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B100">
         <v>6</v>
       </c>
       <c r="C100" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="K100" s="1"/>
     </row>
     <row r="101" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B101">
         <v>7</v>
       </c>
       <c r="C101" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="K101" s="1"/>
     </row>
     <row r="102" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B102">
         <v>8</v>
       </c>
       <c r="C102" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="K102" s="1"/>
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B103">
         <v>9</v>
       </c>
       <c r="C103" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="I103" s="1"/>
       <c r="K103" s="1"/>
     </row>
     <row r="104" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B104">
         <v>10</v>
       </c>
       <c r="C104" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="K104" s="1"/>
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B105">
         <v>11</v>
       </c>
       <c r="C105" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="I105" s="1"/>
       <c r="J105" s="1"/>
@@ -2524,139 +2524,139 @@
     </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B106">
         <v>12</v>
       </c>
       <c r="C106" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="J106" s="1"/>
       <c r="K106" s="1"/>
     </row>
     <row r="107" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B107">
         <v>13</v>
       </c>
       <c r="C107" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="J107" s="1"/>
       <c r="K107" s="1"/>
     </row>
     <row r="108" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B108">
         <v>14</v>
       </c>
       <c r="C108" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="K108" s="1"/>
     </row>
     <row r="109" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B109">
         <v>15</v>
       </c>
       <c r="C109" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="K109" s="1"/>
     </row>
     <row r="110" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B110">
         <v>16</v>
       </c>
       <c r="C110" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="J110" s="1"/>
       <c r="K110" s="1"/>
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B111">
         <v>17</v>
       </c>
       <c r="C111" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="J111" s="1"/>
       <c r="K111" s="1"/>
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B112">
         <v>18</v>
       </c>
       <c r="C112" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="K112" s="1"/>
     </row>
     <row r="113" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B113">
         <v>19</v>
       </c>
       <c r="C113" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="I113" s="1"/>
       <c r="K113" s="1"/>
     </row>
     <row r="114" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B114">
         <v>20</v>
       </c>
       <c r="C114" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="J114" s="1"/>
       <c r="K114" s="1"/>
     </row>
     <row r="115" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B115">
         <v>21</v>
       </c>
       <c r="C115" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="K115" s="1"/>
     </row>
     <row r="116" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B116">
         <v>22</v>
       </c>
       <c r="C116" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="K116" s="1"/>
     </row>
@@ -2990,7 +2990,7 @@
         <v>12</v>
       </c>
       <c r="C143" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="K143" s="1"/>
     </row>
@@ -3038,7 +3038,7 @@
         <v>16</v>
       </c>
       <c r="C147" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="K147" s="1"/>
     </row>
@@ -3068,1024 +3068,1024 @@
     </row>
     <row r="150" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
-        <v>84</v>
+        <v>245</v>
       </c>
       <c r="B150">
         <v>1</v>
       </c>
       <c r="C150" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="K150" s="1"/>
     </row>
     <row r="151" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
-        <v>84</v>
+        <v>245</v>
       </c>
       <c r="B151">
         <v>2</v>
       </c>
       <c r="C151" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="K151" s="1"/>
     </row>
     <row r="152" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
-        <v>84</v>
+        <v>245</v>
       </c>
       <c r="B152">
         <v>3</v>
       </c>
       <c r="C152" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="J152" s="1"/>
       <c r="K152" s="1"/>
     </row>
     <row r="153" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
-        <v>84</v>
+        <v>245</v>
       </c>
       <c r="B153">
         <v>4</v>
       </c>
       <c r="C153" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="K153" s="1"/>
     </row>
     <row r="154" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
-        <v>84</v>
+        <v>245</v>
       </c>
       <c r="B154">
         <v>5</v>
       </c>
       <c r="C154" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K154" s="1"/>
     </row>
     <row r="155" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
-        <v>84</v>
+        <v>245</v>
       </c>
       <c r="B155">
         <v>6</v>
       </c>
       <c r="C155" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I155" s="1"/>
       <c r="K155" s="1"/>
     </row>
     <row r="156" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
-        <v>84</v>
+        <v>245</v>
       </c>
       <c r="B156">
         <v>7</v>
       </c>
       <c r="C156" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J156" s="1"/>
       <c r="K156" s="1"/>
     </row>
     <row r="157" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
-        <v>84</v>
+        <v>245</v>
       </c>
       <c r="B157">
         <v>8</v>
       </c>
       <c r="C157" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="K157" s="1"/>
     </row>
     <row r="158" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
-        <v>84</v>
+        <v>245</v>
       </c>
       <c r="B158">
         <v>9</v>
       </c>
       <c r="C158" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="K158" s="1"/>
     </row>
     <row r="159" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
-        <v>84</v>
+        <v>245</v>
       </c>
       <c r="B159">
         <v>10</v>
       </c>
       <c r="C159" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="K159" s="1"/>
     </row>
     <row r="160" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
-        <v>84</v>
+        <v>245</v>
       </c>
       <c r="B160">
         <v>11</v>
       </c>
       <c r="C160" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="K160" s="1"/>
     </row>
     <row r="161" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
-        <v>84</v>
+        <v>245</v>
       </c>
       <c r="B161">
         <v>12</v>
       </c>
       <c r="C161" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="J161" s="1"/>
       <c r="K161" s="1"/>
     </row>
     <row r="162" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
-        <v>84</v>
+        <v>245</v>
       </c>
       <c r="B162">
         <v>13</v>
       </c>
       <c r="C162" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K162" s="1"/>
     </row>
     <row r="163" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
-        <v>84</v>
+        <v>245</v>
       </c>
       <c r="B163">
         <v>14</v>
       </c>
       <c r="C163" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="K163" s="1"/>
     </row>
     <row r="164" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
-        <v>84</v>
+        <v>245</v>
       </c>
       <c r="B164">
         <v>15</v>
       </c>
       <c r="C164" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J164" s="1"/>
       <c r="K164" s="1"/>
     </row>
     <row r="165" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
-        <v>84</v>
+        <v>245</v>
       </c>
       <c r="B165">
         <v>16</v>
       </c>
       <c r="C165" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K165" s="1"/>
     </row>
     <row r="166" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
-        <v>84</v>
+        <v>245</v>
       </c>
       <c r="B166">
         <v>17</v>
       </c>
       <c r="C166" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="K166" s="1"/>
     </row>
     <row r="167" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
-        <v>100</v>
+        <v>244</v>
       </c>
       <c r="B167">
         <v>1</v>
       </c>
       <c r="C167" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="K167" s="1"/>
     </row>
     <row r="168" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
-        <v>100</v>
+        <v>244</v>
       </c>
       <c r="B168">
         <v>2</v>
       </c>
       <c r="C168" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="K168" s="1"/>
     </row>
     <row r="169" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
-        <v>100</v>
+        <v>244</v>
       </c>
       <c r="B169">
         <v>3</v>
       </c>
       <c r="C169" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="K169" s="1"/>
     </row>
     <row r="170" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
-        <v>100</v>
+        <v>244</v>
       </c>
       <c r="B170">
         <v>4</v>
       </c>
       <c r="C170" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="K170" s="1"/>
     </row>
     <row r="171" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
-        <v>100</v>
+        <v>244</v>
       </c>
       <c r="B171">
         <v>5</v>
       </c>
       <c r="C171" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="K171" s="1"/>
     </row>
     <row r="172" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
-        <v>100</v>
+        <v>244</v>
       </c>
       <c r="B172">
         <v>6</v>
       </c>
       <c r="C172" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="K172" s="1"/>
     </row>
     <row r="173" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
-        <v>100</v>
+        <v>244</v>
       </c>
       <c r="B173">
         <v>7</v>
       </c>
       <c r="C173" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="J173" s="1"/>
       <c r="K173" s="1"/>
     </row>
     <row r="174" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
-        <v>100</v>
+        <v>244</v>
       </c>
       <c r="B174">
         <v>8</v>
       </c>
       <c r="C174" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="K174" s="1"/>
     </row>
     <row r="175" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
-        <v>100</v>
+        <v>244</v>
       </c>
       <c r="B175">
         <v>9</v>
       </c>
       <c r="C175" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="J175" s="1"/>
       <c r="K175" s="1"/>
     </row>
     <row r="176" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
-        <v>100</v>
+        <v>244</v>
       </c>
       <c r="B176">
         <v>10</v>
       </c>
       <c r="C176" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K176" s="1"/>
     </row>
     <row r="177" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
-        <v>100</v>
+        <v>244</v>
       </c>
       <c r="B177">
         <v>11</v>
       </c>
       <c r="C177" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="K177" s="1"/>
     </row>
     <row r="178" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
-        <v>100</v>
+        <v>244</v>
       </c>
       <c r="B178">
         <v>12</v>
       </c>
       <c r="C178" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="K178" s="1"/>
     </row>
     <row r="179" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
-        <v>100</v>
+        <v>244</v>
       </c>
       <c r="B179">
         <v>13</v>
       </c>
       <c r="C179" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="K179" s="1"/>
     </row>
     <row r="180" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
-        <v>100</v>
+        <v>244</v>
       </c>
       <c r="B180">
         <v>14</v>
       </c>
       <c r="C180" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="K180" s="1"/>
     </row>
     <row r="181" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
-        <v>100</v>
+        <v>244</v>
       </c>
       <c r="B181">
         <v>15</v>
       </c>
       <c r="C181" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="I181" s="1"/>
       <c r="K181" s="1"/>
     </row>
     <row r="182" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
-        <v>100</v>
+        <v>244</v>
       </c>
       <c r="B182">
         <v>16</v>
       </c>
       <c r="C182" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="K182" s="1"/>
     </row>
     <row r="183" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
-        <v>100</v>
+        <v>244</v>
       </c>
       <c r="B183">
         <v>17</v>
       </c>
       <c r="C183" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="K183" s="1"/>
     </row>
     <row r="184" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B184">
         <v>1</v>
       </c>
       <c r="C184" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="K184" s="1"/>
     </row>
     <row r="185" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B185">
         <v>2</v>
       </c>
       <c r="C185" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="K185" s="1"/>
     </row>
     <row r="186" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B186">
         <v>3</v>
       </c>
       <c r="C186" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="K186" s="1"/>
     </row>
     <row r="187" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B187">
         <v>4</v>
       </c>
       <c r="C187" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="K187" s="1"/>
     </row>
     <row r="188" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B188">
         <v>5</v>
       </c>
       <c r="C188" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="K188" s="1"/>
     </row>
     <row r="189" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B189">
         <v>6</v>
       </c>
       <c r="C189" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="K189" s="1"/>
     </row>
     <row r="190" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B190">
         <v>7</v>
       </c>
       <c r="C190" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="K190" s="1"/>
     </row>
     <row r="191" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B191">
         <v>8</v>
       </c>
       <c r="C191" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="K191" s="1"/>
     </row>
     <row r="192" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B192">
         <v>9</v>
       </c>
       <c r="C192" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="K192" s="1"/>
     </row>
     <row r="193" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B193">
         <v>10</v>
       </c>
       <c r="C193" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="K193" s="1"/>
     </row>
     <row r="194" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B194">
         <v>11</v>
       </c>
       <c r="C194" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="K194" s="1"/>
     </row>
     <row r="195" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B195">
         <v>12</v>
       </c>
       <c r="C195" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="K195" s="1"/>
     </row>
     <row r="196" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B196">
         <v>13</v>
       </c>
       <c r="C196" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="197" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B197">
         <v>14</v>
       </c>
       <c r="C197" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="198" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B198">
         <v>15</v>
       </c>
       <c r="C198" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="199" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B199">
         <v>16</v>
       </c>
       <c r="C199" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="200" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B200">
         <v>17</v>
       </c>
       <c r="C200" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="201" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B201">
         <v>18</v>
       </c>
       <c r="C201" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="202" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B202">
         <v>19</v>
       </c>
       <c r="C202" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="203" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B203">
         <v>20</v>
       </c>
       <c r="C203" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="204" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B204">
         <v>21</v>
       </c>
       <c r="C204" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="205" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B205">
         <v>22</v>
       </c>
       <c r="C205" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="206" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B206">
         <v>23</v>
       </c>
       <c r="C206" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="207" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B207">
         <v>1</v>
       </c>
       <c r="C207" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="208" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B208">
         <v>2</v>
       </c>
       <c r="C208" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B209">
         <v>3</v>
       </c>
       <c r="C209" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B210">
         <v>4</v>
       </c>
       <c r="C210" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B211">
         <v>5</v>
       </c>
       <c r="C211" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B212">
         <v>6</v>
       </c>
       <c r="C212" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B213">
         <v>7</v>
       </c>
       <c r="C213" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B214">
         <v>8</v>
       </c>
       <c r="C214" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A215" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B215">
         <v>9</v>
       </c>
       <c r="C215" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A216" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B216">
         <v>10</v>
       </c>
       <c r="C216" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A217" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B217">
         <v>11</v>
       </c>
       <c r="C217" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A218" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B218">
         <v>12</v>
       </c>
       <c r="C218" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A219" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B219">
         <v>13</v>
       </c>
       <c r="C219" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A220" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B220">
         <v>14</v>
       </c>
       <c r="C220" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A221" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B221">
         <v>15</v>
       </c>
       <c r="C221" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B222">
         <v>16</v>
       </c>
       <c r="C222" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A223" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B223">
         <v>17</v>
       </c>
       <c r="C223" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B224">
         <v>18</v>
       </c>
       <c r="C224" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B225">
         <v>19</v>
       </c>
       <c r="C225" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B226">
         <v>20</v>
       </c>
       <c r="C226" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B227">
         <v>21</v>
       </c>
       <c r="C227" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B228">
         <v>22</v>
       </c>
       <c r="C228" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B229">
         <v>23</v>
       </c>
       <c r="C229" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B230">
         <v>24</v>
       </c>
       <c r="C230" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B231">
         <v>25</v>
       </c>
       <c r="C231" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B232">
         <v>26</v>
       </c>
       <c r="C232" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B233">
         <v>27</v>
       </c>
       <c r="C233" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B234">
         <v>28</v>
       </c>
       <c r="C234" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A235" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B235">
         <v>29</v>
       </c>
       <c r="C235" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A236" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B236">
         <v>30</v>
       </c>
       <c r="C236" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B237">
         <v>31</v>
       </c>
       <c r="C237" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated excel file and word remove list
Updated the esxcel file for all teh songs with the life of a showgirl. In addition i added (feat. Sabrina Carpenter) to the word-remove list
</commit_message>
<xml_diff>
--- a/excelToJS/taylor_all_album_songs.xlsx
+++ b/excelToJS/taylor_all_album_songs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10309"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stormwinnem/Desktop/Repositories/Swift-Sounds/excelToJS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFDF3E40-1BEB-E14F-8AFE-20B6C328B040}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E058A8FF-BD24-4748-BCBD-1DB6E4D9E780}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{0842053E-6FEE-2E43-A668-BC17E9E71A07}"/>
   </bookViews>
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="259">
   <si>
     <t>album_name</t>
   </si>
@@ -817,6 +817,45 @@
   </si>
   <si>
     <t>folklore (deluxe version)</t>
+  </si>
+  <si>
+    <t>The Life of a Showgirl</t>
+  </si>
+  <si>
+    <t>The Fate of Ophelia</t>
+  </si>
+  <si>
+    <t>Elizabeth Taylor</t>
+  </si>
+  <si>
+    <t>Opalite</t>
+  </si>
+  <si>
+    <t>Father Figure</t>
+  </si>
+  <si>
+    <t>Eldest Daughter</t>
+  </si>
+  <si>
+    <t>Ruin The Friendship</t>
+  </si>
+  <si>
+    <t>Actually Romantic</t>
+  </si>
+  <si>
+    <t>Wi$h Li$t</t>
+  </si>
+  <si>
+    <t>Wood</t>
+  </si>
+  <si>
+    <t>CANCELLED!</t>
+  </si>
+  <si>
+    <t>Honey</t>
+  </si>
+  <si>
+    <t>The Life of a Showgirl (feat. Sabrina Carpenter)</t>
   </si>
 </sst>
 </file>
@@ -1199,7 +1238,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1641E2E9-0811-C947-A1BC-4F111B0518AB}">
-  <dimension ref="A1:K237"/>
+  <dimension ref="A1:K249"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="45" customWidth="1"/>
@@ -4088,6 +4127,138 @@
         <v>241</v>
       </c>
     </row>
+    <row r="238" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A238" t="s">
+        <v>246</v>
+      </c>
+      <c r="B238">
+        <v>1</v>
+      </c>
+      <c r="C238" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="239" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A239" t="s">
+        <v>246</v>
+      </c>
+      <c r="B239">
+        <v>2</v>
+      </c>
+      <c r="C239" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="240" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A240" t="s">
+        <v>246</v>
+      </c>
+      <c r="B240">
+        <v>3</v>
+      </c>
+      <c r="C240" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="241" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A241" t="s">
+        <v>246</v>
+      </c>
+      <c r="B241">
+        <v>4</v>
+      </c>
+      <c r="C241" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="242" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A242" t="s">
+        <v>246</v>
+      </c>
+      <c r="B242">
+        <v>5</v>
+      </c>
+      <c r="C242" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="243" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A243" t="s">
+        <v>246</v>
+      </c>
+      <c r="B243">
+        <v>6</v>
+      </c>
+      <c r="C243" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="244" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A244" t="s">
+        <v>246</v>
+      </c>
+      <c r="B244">
+        <v>7</v>
+      </c>
+      <c r="C244" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="245" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A245" t="s">
+        <v>246</v>
+      </c>
+      <c r="B245">
+        <v>8</v>
+      </c>
+      <c r="C245" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="246" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A246" t="s">
+        <v>246</v>
+      </c>
+      <c r="B246">
+        <v>9</v>
+      </c>
+      <c r="C246" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="247" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A247" t="s">
+        <v>246</v>
+      </c>
+      <c r="B247">
+        <v>10</v>
+      </c>
+      <c r="C247" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="248" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A248" t="s">
+        <v>246</v>
+      </c>
+      <c r="B248">
+        <v>11</v>
+      </c>
+      <c r="C248" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="249" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A249" t="s">
+        <v>246</v>
+      </c>
+      <c r="B249">
+        <v>12</v>
+      </c>
+      <c r="C249" t="s">
+        <v>258</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>